<commit_message>
Add Relative Valuation (comps) sheet
Comparable company analysis (TVS, Bajaj, Hero, Eicher, Ola Electric vs Ather) with EV/Sales, EV/EBITDA, P/E; EV/Sales-based implied value for Ather and a football field vs DCF and current market price.
</commit_message>
<xml_diff>
--- a/Ather_Financial_Model.xlsx
+++ b/Ather_Financial_Model.xlsx
@@ -19,8 +19,9 @@
     <sheet name="Ratio Analysis" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Error Checks" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="DCF" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Company &amp; Market Insights" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Modelling Notes" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Relative Valuation" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Company &amp; Market Insights" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Modelling Notes" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -184,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -341,6 +342,36 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -3872,6 +3903,607 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="007030A0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:O33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2.5" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Ather Energy Ltd — Relative Valuation (Comparable Companies)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="B3" s="54" t="inlineStr">
+        <is>
+          <t>Peer market data indicative, as of ~Jun-2026 (public sources: NSE/BSE, stockanalysis, dhan, companies-marketcap). Figures in INR crore unless stated. 1 cr = 10 INR m.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="B5" s="55" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C5" s="55" t="inlineStr">
+        <is>
+          <t>Mkt cap (cr)</t>
+        </is>
+      </c>
+      <c r="D5" s="55" t="inlineStr">
+        <is>
+          <t>Net debt (cr)</t>
+        </is>
+      </c>
+      <c r="E5" s="55" t="inlineStr">
+        <is>
+          <t>EV (cr)</t>
+        </is>
+      </c>
+      <c r="F5" s="55" t="inlineStr">
+        <is>
+          <t>Revenue (cr)</t>
+        </is>
+      </c>
+      <c r="G5" s="55" t="inlineStr">
+        <is>
+          <t>EBITDA (cr)</t>
+        </is>
+      </c>
+      <c r="H5" s="55" t="inlineStr">
+        <is>
+          <t>PAT (cr)</t>
+        </is>
+      </c>
+      <c r="I5" s="55" t="inlineStr">
+        <is>
+          <t>EV/Sales</t>
+        </is>
+      </c>
+      <c r="J5" s="55" t="inlineStr">
+        <is>
+          <t>EV/EBITDA</t>
+        </is>
+      </c>
+      <c r="K5" s="55" t="inlineStr">
+        <is>
+          <t>P/E</t>
+        </is>
+      </c>
+      <c r="L5" s="55" t="inlineStr">
+        <is>
+          <t>EBITDA %</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>TVS Motor</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="n">
+        <v>169592</v>
+      </c>
+      <c r="D6" s="28" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E6" s="56">
+        <f>C6+D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="28" t="n">
+        <v>36000</v>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>4320</v>
+      </c>
+      <c r="H6" s="28" t="n">
+        <v>2200</v>
+      </c>
+      <c r="I6" s="44">
+        <f>E6/F6</f>
+        <v/>
+      </c>
+      <c r="J6" s="44">
+        <f>IF(G6&gt;0,E6/G6,"NM")</f>
+        <v/>
+      </c>
+      <c r="K6" s="44">
+        <f>IF(H6&gt;0,C6/H6,"NM")</f>
+        <v/>
+      </c>
+      <c r="L6" s="37">
+        <f>G6/F6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Bajaj Auto</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="n">
+        <v>265000</v>
+      </c>
+      <c r="D7" s="28" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="E7" s="56">
+        <f>C7+D7</f>
+        <v/>
+      </c>
+      <c r="F7" s="28" t="n">
+        <v>49000</v>
+      </c>
+      <c r="G7" s="28" t="n">
+        <v>9800</v>
+      </c>
+      <c r="H7" s="28" t="n">
+        <v>7300</v>
+      </c>
+      <c r="I7" s="44">
+        <f>E7/F7</f>
+        <v/>
+      </c>
+      <c r="J7" s="44">
+        <f>IF(G7&gt;0,E7/G7,"NM")</f>
+        <v/>
+      </c>
+      <c r="K7" s="44">
+        <f>IF(H7&gt;0,C7/H7,"NM")</f>
+        <v/>
+      </c>
+      <c r="L7" s="37">
+        <f>G7/F7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Hero MotoCorp</t>
+        </is>
+      </c>
+      <c r="C8" s="28" t="n">
+        <v>90000</v>
+      </c>
+      <c r="D8" s="28" t="n">
+        <v>-8000</v>
+      </c>
+      <c r="E8" s="56">
+        <f>C8+D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="28" t="n">
+        <v>40000</v>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>5600</v>
+      </c>
+      <c r="H8" s="28" t="n">
+        <v>4500</v>
+      </c>
+      <c r="I8" s="44">
+        <f>E8/F8</f>
+        <v/>
+      </c>
+      <c r="J8" s="44">
+        <f>IF(G8&gt;0,E8/G8,"NM")</f>
+        <v/>
+      </c>
+      <c r="K8" s="44">
+        <f>IF(H8&gt;0,C8/H8,"NM")</f>
+        <v/>
+      </c>
+      <c r="L8" s="37">
+        <f>G8/F8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Eicher Motors</t>
+        </is>
+      </c>
+      <c r="C9" s="28" t="n">
+        <v>208424</v>
+      </c>
+      <c r="D9" s="28" t="n">
+        <v>-16000</v>
+      </c>
+      <c r="E9" s="56">
+        <f>C9+D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="28" t="n">
+        <v>18000</v>
+      </c>
+      <c r="G9" s="28" t="n">
+        <v>4500</v>
+      </c>
+      <c r="H9" s="28" t="n">
+        <v>4700</v>
+      </c>
+      <c r="I9" s="44">
+        <f>E9/F9</f>
+        <v/>
+      </c>
+      <c r="J9" s="44">
+        <f>IF(G9&gt;0,E9/G9,"NM")</f>
+        <v/>
+      </c>
+      <c r="K9" s="44">
+        <f>IF(H9&gt;0,C9/H9,"NM")</f>
+        <v/>
+      </c>
+      <c r="L9" s="37">
+        <f>G9/F9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Ola Electric</t>
+        </is>
+      </c>
+      <c r="C10" s="28" t="n">
+        <v>19000</v>
+      </c>
+      <c r="D10" s="28" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="E10" s="56">
+        <f>C10+D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="28" t="n">
+        <v>4514</v>
+      </c>
+      <c r="G10" s="28" t="n">
+        <v>-1500</v>
+      </c>
+      <c r="H10" s="28" t="n">
+        <v>-2000</v>
+      </c>
+      <c r="I10" s="44">
+        <f>E10/F10</f>
+        <v/>
+      </c>
+      <c r="J10" s="44">
+        <f>IF(G10&gt;0,E10/G10,"NM")</f>
+        <v/>
+      </c>
+      <c r="K10" s="44">
+        <f>IF(H10&gt;0,C10/H10,"NM")</f>
+        <v/>
+      </c>
+      <c r="L10" s="37">
+        <f>G10/F10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Ather Energy (mkt)</t>
+        </is>
+      </c>
+      <c r="C11" s="28" t="n">
+        <v>37920</v>
+      </c>
+      <c r="D11" s="28" t="n">
+        <v>150</v>
+      </c>
+      <c r="E11" s="56">
+        <f>C11+D11</f>
+        <v/>
+      </c>
+      <c r="F11" s="28" t="n">
+        <v>2255</v>
+      </c>
+      <c r="G11" s="28" t="n">
+        <v>-581</v>
+      </c>
+      <c r="H11" s="28" t="n">
+        <v>-812</v>
+      </c>
+      <c r="I11" s="44">
+        <f>E11/F11</f>
+        <v/>
+      </c>
+      <c r="J11" s="44">
+        <f>IF(G11&gt;0,E11/G11,"NM")</f>
+        <v/>
+      </c>
+      <c r="K11" s="44">
+        <f>IF(H11&gt;0,C11/H11,"NM")</f>
+        <v/>
+      </c>
+      <c r="L11" s="37">
+        <f>G11/F11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Legacy 2W OEM median (TVS/Bajaj/Hero/Eicher)</t>
+        </is>
+      </c>
+      <c r="I13" s="57">
+        <f>MEDIAN(I6:I9)</f>
+        <v/>
+      </c>
+      <c r="J13" s="57">
+        <f>MEDIAN(J6:J9)</f>
+        <v/>
+      </c>
+      <c r="K13" s="57">
+        <f>MEDIAN(K6:K9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>EV pure-play reference (Ola Electric)</t>
+        </is>
+      </c>
+      <c r="I14" s="57">
+        <f>I10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>Implied valuation of Ather Energy (EV/Sales — primary, as company is pre-profit)</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="n"/>
+      <c r="D16" s="20" t="n"/>
+      <c r="E16" s="20" t="n"/>
+      <c r="F16" s="20" t="n"/>
+      <c r="G16" s="20" t="n"/>
+      <c r="H16" s="20" t="n"/>
+      <c r="I16" s="20" t="n"/>
+      <c r="J16" s="20" t="n"/>
+      <c r="K16" s="20" t="n"/>
+      <c r="L16" s="20" t="n"/>
+      <c r="M16" s="20" t="n"/>
+      <c r="N16" s="20" t="n"/>
+      <c r="O16" s="20" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Ather FY2027E revenue (INR cr)</t>
+        </is>
+      </c>
+      <c r="C17" s="32">
+        <f>PL!I5/10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Ather net debt — FY2025 (INR cr)</t>
+        </is>
+      </c>
+      <c r="C18" s="32">
+        <f>(BS!G13+BS!G21+BS!G14+BS!G22-BS!G43)/10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Shares outstanding (m)</t>
+        </is>
+      </c>
+      <c r="C19" s="28" t="n">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="C21" s="58" t="inlineStr">
+        <is>
+          <t>EV/Sales (x)</t>
+        </is>
+      </c>
+      <c r="D21" s="58" t="inlineStr">
+        <is>
+          <t>Implied EV (cr)</t>
+        </is>
+      </c>
+      <c r="E21" s="58" t="inlineStr">
+        <is>
+          <t>Implied equity (cr)</t>
+        </is>
+      </c>
+      <c r="F21" s="58" t="inlineStr">
+        <is>
+          <t>Implied price (INR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Conservative (3.0x)</t>
+        </is>
+      </c>
+      <c r="C22" s="59" t="n">
+        <v>3</v>
+      </c>
+      <c r="D22" s="56">
+        <f>C22*$C$17</f>
+        <v/>
+      </c>
+      <c r="E22" s="56">
+        <f>D22-$C$18</f>
+        <v/>
+      </c>
+      <c r="F22" s="60">
+        <f>E22*10/$C$19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Base (4.5x)</t>
+        </is>
+      </c>
+      <c r="C23" s="59" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D23" s="56">
+        <f>C23*$C$17</f>
+        <v/>
+      </c>
+      <c r="E23" s="56">
+        <f>D23-$C$18</f>
+        <v/>
+      </c>
+      <c r="F23" s="60">
+        <f>E23*10/$C$19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Bull (6.0x)</t>
+        </is>
+      </c>
+      <c r="C24" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="D24" s="56">
+        <f>C24*$C$17</f>
+        <v/>
+      </c>
+      <c r="E24" s="56">
+        <f>D24-$C$18</f>
+        <v/>
+      </c>
+      <c r="F24" s="60">
+        <f>E24*10/$C$19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="19" t="inlineStr">
+        <is>
+          <t>Valuation summary (football field)</t>
+        </is>
+      </c>
+      <c r="C27" s="20" t="n"/>
+      <c r="D27" s="20" t="n"/>
+      <c r="E27" s="20" t="n"/>
+      <c r="F27" s="20" t="n"/>
+      <c r="G27" s="20" t="n"/>
+      <c r="H27" s="20" t="n"/>
+      <c r="I27" s="20" t="n"/>
+      <c r="J27" s="20" t="n"/>
+      <c r="K27" s="20" t="n"/>
+      <c r="L27" s="20" t="n"/>
+      <c r="M27" s="20" t="n"/>
+      <c r="N27" s="20" t="n"/>
+      <c r="O27" s="20" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>DCF — Base case (INR/share)</t>
+        </is>
+      </c>
+      <c r="C28" s="61">
+        <f>DCF!C27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Relative — conservative to bull (INR/share)</t>
+        </is>
+      </c>
+      <c r="C29" s="60">
+        <f>F22</f>
+        <v/>
+      </c>
+      <c r="D29" s="7">
+        <f>"to "&amp;TEXT(F24,"#,##0")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Current market price (INR/share)</t>
+        </is>
+      </c>
+      <c r="C30" s="62" t="n">
+        <v>990</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Implied market EV/Sales on FY25 revenue (x)</t>
+        </is>
+      </c>
+      <c r="C31" s="63">
+        <f>I11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="58" customHeight="1">
+      <c r="B33" s="54" t="inlineStr">
+        <is>
+          <t>Read-through: Ather trades at a steep premium to legacy 2W OEMs and to Ola Electric on EV/Sales, so the market is already pricing in strong volume growth and a sharp margin ramp. On a conservative DCF and on peer-based EV/Sales, the stock screens expensive unless one underwrites the bull-case volumes and terminal margins. Use this alongside the DCF and the Scenarios switch. Indicative, not investment advice.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00808080"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -3891,112 +4523,112 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="B4" s="54" t="inlineStr">
+      <c r="B4" s="64" t="inlineStr">
         <is>
           <t>Company snapshot</t>
         </is>
       </c>
     </row>
     <row r="5" ht="60" customHeight="1">
-      <c r="B5" s="55" t="inlineStr">
+      <c r="B5" s="65" t="inlineStr">
         <is>
           <t>Ather Energy Ltd (Bengaluru; incorporated 2013) designs and manufactures premium smart electric scooters (450 series, Rizta) and runs the AtherStack software and Ather Grid charging ecosystem. It listed on NSE/BSE in May 2025. Ather prepares STANDALONE financial statements only — it has no subsidiaries, so no consolidated statements exist; standalone is therefore the consolidated-equivalent used here.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="B6" s="54" t="inlineStr">
+      <c r="B6" s="64" t="inlineStr">
         <is>
           <t>Operating performance</t>
         </is>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1">
-      <c r="B7" s="55" t="inlineStr">
+      <c r="B7" s="65" t="inlineStr">
         <is>
           <t>Revenue grew from INR 798m (FY21) to INR 22,550m (FY25); FY25 revenue +29% YoY. The company remains loss-making (FY25 PAT INR -8,123m) but gross margin inflected sharply to ~16.8% in FY25 (from ~7% FY24) on scale, the Rizta launch and falling battery costs. Vehicle sales are ~88% of revenue; software, accessories, charging and service make up the balance and are higher-margin, recurring streams.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="B8" s="54" t="inlineStr">
+      <c r="B8" s="64" t="inlineStr">
         <is>
           <t>Volumes, ASP &amp; market share</t>
         </is>
       </c>
     </row>
     <row r="9" ht="60" customHeight="1">
-      <c r="B9" s="55" t="inlineStr">
+      <c r="B9" s="65" t="inlineStr">
         <is>
           <t>FY25 deliveries ~1.65 lakh units; revenue per vehicle ~INR 1.28 lakh (down from ~1.43 lakh FY24 and ~1.56 lakh FY23 as the cheaper Rizta lifted mix). Ather's E2W market share rose from ~13-14% (FY25) to ~18.7% by Mar-2026; retail network expanded from 351 outlets (Mar-25) toward ~700 (FY26). Source: Vahan / ETAuto / Autocar India / Storyboard18.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="B10" s="54" t="inlineStr">
+      <c r="B10" s="64" t="inlineStr">
         <is>
           <t>Industry &amp; demand drivers</t>
         </is>
       </c>
     </row>
     <row r="11" ht="60" customHeight="1">
-      <c r="B11" s="55" t="inlineStr">
+      <c r="B11" s="65" t="inlineStr">
         <is>
           <t>India electric two-wheeler volumes (~1.1-1.2m in FY25) are forecast to grow ~26-28% CAGR to 2034 (IMARC/Renub/TechSci). E2W penetration of the ~19m-unit 2W market is ~6-7% today and is projected at ~30% by 2030 (Kearney) and up to ~40% by FY31 in Ather's optimistic case. PM E-DRIVE (successor to FAME-II), 5% GST on EVs, state EV policies and PLI for cell manufacturing support demand and localisation.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="B12" s="54" t="inlineStr">
+      <c r="B12" s="64" t="inlineStr">
         <is>
           <t>Battery cost trend (key margin lever)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="45" customHeight="1">
-      <c r="B13" s="55" t="inlineStr">
+      <c r="B13" s="65" t="inlineStr">
         <is>
           <t>Lithium-ion pack prices fell ~8% to ~USD 108/kWh in 2025 and are forecast at ~USD 105/kWh in 2026, declining toward ~USD 80-90/kWh by 2030 (BloombergNEF, Dec-2025), aided by cell overcapacity and an ~84% lithium price correction. Batteries are Ather's largest input cost, so this is a structural gross-margin tailwind.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
-      <c r="B14" s="54" t="inlineStr">
+      <c r="B14" s="64" t="inlineStr">
         <is>
           <t>Competition</t>
         </is>
       </c>
     </row>
     <row r="15" ht="60" customHeight="1">
-      <c r="B15" s="55" t="inlineStr">
+      <c r="B15" s="65" t="inlineStr">
         <is>
           <t>Top E2W OEMs (CY2025 / early-2026 Vahan): TVS Motor ~24%, Bajaj Auto ~22%, Ather ~13-18%, with Ola Electric's share collapsing (24.8% Jan-25 to &lt;6% Jan-26), plus Hero/Greaves. TVS and Bajaj are profitable legacy OEMs with large ICE dealer networks; Ola and Ather are pure-play EV challengers still investing for scale. Ather differentiates on software, design and a premium brand.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="B16" s="54" t="inlineStr">
+      <c r="B16" s="64" t="inlineStr">
         <is>
           <t>Capital &amp; capacity</t>
         </is>
       </c>
     </row>
     <row r="17" ht="45" customHeight="1">
-      <c r="B17" s="55" t="inlineStr">
+      <c r="B17" s="65" t="inlineStr">
         <is>
           <t>The IPO raised a fresh issue of ~INR 2,626 cr (~26,260m), used for the new Maharashtra plant (Factory-3, tripling capacity), R&amp;D, debt repayment and marketing. Post-IPO shares outstanding ~372m. Large accumulated tax losses (&gt;INR 40,000m) shield taxable income across the forecast horizon (statutory rate 25.17%).</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="B18" s="54" t="inlineStr">
+      <c r="B18" s="64" t="inlineStr">
         <is>
           <t>Sources</t>
         </is>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
-      <c r="B19" s="56" t="inlineStr">
+      <c r="B19" s="66" t="inlineStr">
         <is>
           <t>BloombergNEF battery price survey (Dec-2025); SIAM / Vahan registration data; ETAuto, Economic Times, Moneycontrol, Autocar India, Storyboard18, Angel One, Financial Express; IMARC / Renub / TechSci / Kearney industry reports; Ather Energy Annual Reports FY2021-FY2025 (standalone financial statements). Content paraphrased / summarised for licensing compliance.</t>
         </is>
@@ -4007,7 +4639,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00808080"/>
@@ -4029,140 +4661,140 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="B4" s="57" t="inlineStr">
+      <c r="B4" s="67" t="inlineStr">
         <is>
           <t>1. Purpose &amp; scope</t>
         </is>
       </c>
     </row>
     <row r="5" ht="60" customHeight="1">
-      <c r="B5" s="55" t="inlineStr">
+      <c r="B5" s="65" t="inlineStr">
         <is>
           <t>Fully-linked, driver-based operating model and DCF for Ather Energy Ltd. History FY2021-FY2025; forecast FY2026E-FY2033E (8 years). All figures INR millions unless stated. Built to mirror the supplied United Spirits template's structure, colour coding and philosophy. Colour key: BLUE = hardcoded input, GREEN = link/reference to another sheet, BLACK = in-sheet calculation.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="B6" s="57" t="inlineStr">
+      <c r="B6" s="67" t="inlineStr">
         <is>
           <t>2. Data basis (consolidated vs standalone)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="105" customHeight="1">
-      <c r="B7" s="55" t="inlineStr">
+      <c r="B7" s="65" t="inlineStr">
         <is>
           <t>Ather has no subsidiaries and files only STANDALONE Ind AS financial statements; no consolidated statements exist, so standalone is used as the consolidated-equivalent. FY2021/22/24/25 are taken directly from the annual reports in the repository. FY2023's annual reports in the repo are image-only (no text layer); FY2023 was therefore reconstructed from reliable public sources (Economic Times/Moneycontrol: revenue INR 17,836m, total expenses INR 26,706m, net loss INR 8,645m, D&amp;A INR 1,128m) and from anchors verified in the FY2025 report (1-Apr-2023 reserves INR 6,131m; opening borrowings/lease; opening cash INR 826m; FY23 inventory INR 2,574m). FY2023 sub-line splits are estimates that reconcile exactly to the verified totals.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="B8" s="57" t="inlineStr">
+      <c r="B8" s="67" t="inlineStr">
         <is>
           <t>3. Revenue methodology</t>
         </is>
       </c>
     </row>
     <row r="9" ht="90" customHeight="1">
-      <c r="B9" s="55" t="inlineStr">
+      <c r="B9" s="65" t="inlineStr">
         <is>
           <t>Driver-based: vehicle revenue = unit volumes x ASP. Volume growth is set on the Scenarios sheet (Base/Bull/Bear) reflecting E2W market growth plus Ather share gains, tapering over time. ASP reflects the recent Rizta-led mix dip then modest premiumisation. Accessories, software/connectivity and charging are forecast as a % of vehicle revenue (higher-margin recurring streams broken out prospectively); service grows with the installed fleet. Historically these streams were bundled into product/service revenue per Note 20, so a small step-up appears in FY2026.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="B10" s="57" t="inlineStr">
+      <c r="B10" s="67" t="inlineStr">
         <is>
           <t>4. Cost, margin &amp; operating leverage</t>
         </is>
       </c>
     </row>
     <row r="11" ht="75" customHeight="1">
-      <c r="B11" s="55" t="inlineStr">
+      <c r="B11" s="65" t="inlineStr">
         <is>
           <t>Gross margin (Scenarios) expands from ~18% (FY26) to ~28% (FY33) on falling battery costs, scale, localisation/PLI and mix. Employee and other operating expenses are forecast as a declining % of sales, capturing operating leverage as a largely fixed cost base is spread over a fast-growing top line. The model reaches EBITDA breakeven around FY2030 and approaches PAT breakeven by FY2032-FY2033 — a realistic path, neither over-optimistic nor over-pessimistic.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="B12" s="57" t="inlineStr">
+      <c r="B12" s="67" t="inlineStr">
         <is>
           <t>5. Schedules</t>
         </is>
       </c>
     </row>
     <row r="13" ht="75" customHeight="1">
-      <c r="B13" s="55" t="inlineStr">
+      <c r="B13" s="65" t="inlineStr">
         <is>
           <t>PPE, ROU (leases) and intangibles use opening + additions - depreciation/amortisation roll-forwards (capex and additions driven off revenue). Depreciation uses a straight-line life with a half-year convention on additions. Borrowings and leases use opening + net movement roll-forwards with interest on opening balances feeding the finance-cost schedule. A tax schedule tracks carry-forward losses (&gt;INR 40,000m) which keep cash tax at nil across the forecast.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
-      <c r="B14" s="57" t="inlineStr">
+      <c r="B14" s="67" t="inlineStr">
         <is>
           <t>6. Integration &amp; balancing</t>
         </is>
       </c>
     </row>
     <row r="15" ht="75" customHeight="1">
-      <c r="B15" s="55" t="inlineStr">
+      <c r="B15" s="65" t="inlineStr">
         <is>
           <t>The three statements are fully linked with no circular references (interest income/expense use opening balances). The model is FULLY ARTICULATED: every balance-sheet line is forecast from a driver and cash is the genuine output of the cash-flow statement, so the balance sheet balances by accounting identity (no balancing plug). The Error Checks sheet confirms balance-sheet balancing, cash-flow reconciliation, beginning/ending balances and all roll-forwards return PASS for every year.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="B16" s="57" t="inlineStr">
+      <c r="B16" s="67" t="inlineStr">
         <is>
           <t>7. Valuation</t>
         </is>
       </c>
     </row>
     <row r="17" ht="60" customHeight="1">
-      <c r="B17" s="55" t="inlineStr">
+      <c r="B17" s="65" t="inlineStr">
         <is>
           <t>An FCFF DCF discounts unlevered free cash flow at a CAPM-based WACC (Rf 6.8%, ERP 5.2%, beta 1.15 -&gt; ~12.8%), with a 5% terminal growth rate. Because Ather is pre-profit, early FCFF is negative and most value sits in the terminal year; the DCF should be read alongside relative valuation (EV/Sales) and the Base/Bull/Bear scenarios.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="B18" s="57" t="inlineStr">
+      <c r="B18" s="67" t="inlineStr">
         <is>
           <t>8. Key risks</t>
         </is>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
-      <c r="B19" s="55" t="inlineStr">
+      <c r="B19" s="65" t="inlineStr">
         <is>
           <t>Demand/competition: aggressive pricing by Ola, TVS, Bajaj could cap volumes/ASP and margins. Margin: slower battery-cost decline or input inflation. Execution: Factory-3 ramp and capex discipline. Funding: the model shows cash thinning by FY2033 — a further capital raise or faster profitability may be required. Policy: changes to PM E-DRIVE/GST incentives. Technology: rare-earth magnet supply and battery-chemistry shifts.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
-      <c r="B20" s="57" t="inlineStr">
+      <c r="B20" s="67" t="inlineStr">
         <is>
           <t>9. Limitations</t>
         </is>
       </c>
     </row>
     <row r="21" ht="60" customHeight="1">
-      <c r="B21" s="55" t="inlineStr">
+      <c r="B21" s="65" t="inlineStr">
         <is>
           <t>FY2023 sub-line items are reconstructed (totals verified). Forecasts are scenario-based judgements, not guidance. Other non-current/other current items are modelled as ratios of sales. The DCF is sensitive to WACC and terminal growth (a sensitivity grid can be layered on). This model is for analytical/educational purposes and is not investment advice.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
-      <c r="B22" s="57" t="inlineStr">
+      <c r="B22" s="67" t="inlineStr">
         <is>
           <t>10. How to use</t>
         </is>
       </c>
     </row>
     <row r="23" ht="45" customHeight="1">
-      <c r="B23" s="55" t="inlineStr">
+      <c r="B23" s="65" t="inlineStr">
         <is>
           <t>Change the single Scenarios!F4 switch (1=Base, 2=Bull, 3=Bear) to flex volume growth and gross margin across the whole model. All other assumptions live on the Assumptions sheet (each with a Source and a plain-language Reason). Inputs are blue; do not type over green links or black formulas.</t>
         </is>

</xml_diff>

<commit_message>
Convert DCF to 3-stage model (explicit FY26-33 + fade FY34-40 + terminal)
Stage 2 fade lets growth converge and EBIT margin ramp to a mature ~15% with taxed NOPAT and reinvestment, so terminal value is struck on a steady-state business rather than a still-immature FY2033. Validated: all checks PASS, no formula errors.
</commit_message>
<xml_diff>
--- a/Ather_Financial_Model.xlsx
+++ b/Ather_Financial_Model.xlsx
@@ -185,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -342,6 +342,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -919,7 +922,7 @@
         </is>
       </c>
       <c r="H12" s="10">
-        <f>DCF!C27</f>
+        <f>DCF!C38</f>
         <v/>
       </c>
     </row>
@@ -3261,11 +3264,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N29"/>
+  <dimension ref="B2:O42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
@@ -3283,7 +3286,7 @@
     <row r="2">
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>Ather Energy Ltd — DCF Valuation (FCFF)</t>
+          <t>Ather Energy Ltd — DCF Valuation (3-stage FCFF)</t>
         </is>
       </c>
       <c r="L2" s="49" t="inlineStr">
@@ -3291,6 +3294,26 @@
           <t>WACC (CAPM)</t>
         </is>
       </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>Stage 1 — Explicit forecast (FY2026E–FY2033E), linked to the detailed model</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="n"/>
+      <c r="D3" s="20" t="n"/>
+      <c r="E3" s="20" t="n"/>
+      <c r="F3" s="20" t="n"/>
+      <c r="G3" s="20" t="n"/>
+      <c r="H3" s="20" t="n"/>
+      <c r="I3" s="20" t="n"/>
+      <c r="J3" s="20" t="n"/>
+      <c r="K3" s="20" t="n"/>
+      <c r="L3" s="20" t="n"/>
+      <c r="M3" s="20" t="n"/>
+      <c r="N3" s="20" t="n"/>
+      <c r="O3" s="20" t="n"/>
     </row>
     <row r="4">
       <c r="B4" s="21" t="inlineStr">
@@ -3344,6 +3367,43 @@
       </c>
     </row>
     <row r="5">
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>EBIT</t>
+        </is>
+      </c>
+      <c r="C5" s="34">
+        <f>PL!H14</f>
+        <v/>
+      </c>
+      <c r="D5" s="34">
+        <f>PL!I14</f>
+        <v/>
+      </c>
+      <c r="E5" s="34">
+        <f>PL!J14</f>
+        <v/>
+      </c>
+      <c r="F5" s="34">
+        <f>PL!K14</f>
+        <v/>
+      </c>
+      <c r="G5" s="34">
+        <f>PL!L14</f>
+        <v/>
+      </c>
+      <c r="H5" s="34">
+        <f>PL!M14</f>
+        <v/>
+      </c>
+      <c r="I5" s="34">
+        <f>PL!N14</f>
+        <v/>
+      </c>
+      <c r="J5" s="34">
+        <f>PL!O14</f>
+        <v/>
+      </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
           <t>Equity market return (Rm)</t>
@@ -3361,39 +3421,39 @@
     <row r="6">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>EBIT</t>
-        </is>
-      </c>
-      <c r="C6" s="34">
-        <f>PL!H14</f>
-        <v/>
-      </c>
-      <c r="D6" s="34">
-        <f>PL!I14</f>
-        <v/>
-      </c>
-      <c r="E6" s="34">
-        <f>PL!J14</f>
-        <v/>
-      </c>
-      <c r="F6" s="34">
-        <f>PL!K14</f>
-        <v/>
-      </c>
-      <c r="G6" s="34">
-        <f>PL!L14</f>
-        <v/>
-      </c>
-      <c r="H6" s="34">
-        <f>PL!M14</f>
-        <v/>
-      </c>
-      <c r="I6" s="34">
-        <f>PL!N14</f>
-        <v/>
-      </c>
-      <c r="J6" s="34">
-        <f>PL!O14</f>
+          <t>Less: tax on EBIT</t>
+        </is>
+      </c>
+      <c r="C6" s="39">
+        <f>-C5*Assumptions!H47</f>
+        <v/>
+      </c>
+      <c r="D6" s="39">
+        <f>-D5*Assumptions!I47</f>
+        <v/>
+      </c>
+      <c r="E6" s="39">
+        <f>-E5*Assumptions!J47</f>
+        <v/>
+      </c>
+      <c r="F6" s="39">
+        <f>-F5*Assumptions!K47</f>
+        <v/>
+      </c>
+      <c r="G6" s="39">
+        <f>-G5*Assumptions!L47</f>
+        <v/>
+      </c>
+      <c r="H6" s="39">
+        <f>-H5*Assumptions!M47</f>
+        <v/>
+      </c>
+      <c r="I6" s="39">
+        <f>-I5*Assumptions!N47</f>
+        <v/>
+      </c>
+      <c r="J6" s="39">
+        <f>-J5*Assumptions!O47</f>
         <v/>
       </c>
       <c r="L6" s="7" t="inlineStr">
@@ -3412,41 +3472,41 @@
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Less: tax on EBIT</t>
-        </is>
-      </c>
-      <c r="C7" s="39">
-        <f>-C6*Assumptions!H47</f>
-        <v/>
-      </c>
-      <c r="D7" s="39">
-        <f>-D6*Assumptions!I47</f>
-        <v/>
-      </c>
-      <c r="E7" s="39">
-        <f>-E6*Assumptions!J47</f>
-        <v/>
-      </c>
-      <c r="F7" s="39">
-        <f>-F6*Assumptions!K47</f>
-        <v/>
-      </c>
-      <c r="G7" s="39">
-        <f>-G6*Assumptions!L47</f>
-        <v/>
-      </c>
-      <c r="H7" s="39">
-        <f>-H6*Assumptions!M47</f>
-        <v/>
-      </c>
-      <c r="I7" s="39">
-        <f>-I6*Assumptions!N47</f>
-        <v/>
-      </c>
-      <c r="J7" s="39">
-        <f>-J6*Assumptions!O47</f>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>NOPAT</t>
+        </is>
+      </c>
+      <c r="C7" s="33">
+        <f>C5+C6</f>
+        <v/>
+      </c>
+      <c r="D7" s="33">
+        <f>D5+D6</f>
+        <v/>
+      </c>
+      <c r="E7" s="33">
+        <f>E5+E6</f>
+        <v/>
+      </c>
+      <c r="F7" s="33">
+        <f>F5+F6</f>
+        <v/>
+      </c>
+      <c r="G7" s="33">
+        <f>G5+G6</f>
+        <v/>
+      </c>
+      <c r="H7" s="33">
+        <f>H5+H6</f>
+        <v/>
+      </c>
+      <c r="I7" s="33">
+        <f>I5+I6</f>
+        <v/>
+      </c>
+      <c r="J7" s="33">
+        <f>J5+J6</f>
         <v/>
       </c>
       <c r="L7" s="7" t="inlineStr">
@@ -3464,41 +3524,41 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>NOPAT</t>
-        </is>
-      </c>
-      <c r="C8" s="33">
-        <f>C6+C7</f>
-        <v/>
-      </c>
-      <c r="D8" s="33">
-        <f>D6+D7</f>
-        <v/>
-      </c>
-      <c r="E8" s="33">
-        <f>E6+E7</f>
-        <v/>
-      </c>
-      <c r="F8" s="33">
-        <f>F6+F7</f>
-        <v/>
-      </c>
-      <c r="G8" s="33">
-        <f>G6+G7</f>
-        <v/>
-      </c>
-      <c r="H8" s="33">
-        <f>H6+H7</f>
-        <v/>
-      </c>
-      <c r="I8" s="33">
-        <f>I6+I7</f>
-        <v/>
-      </c>
-      <c r="J8" s="33">
-        <f>J6+J7</f>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Add: Depreciation &amp; amortisation</t>
+        </is>
+      </c>
+      <c r="C8" s="34">
+        <f>-PL!H13</f>
+        <v/>
+      </c>
+      <c r="D8" s="34">
+        <f>-PL!I13</f>
+        <v/>
+      </c>
+      <c r="E8" s="34">
+        <f>-PL!J13</f>
+        <v/>
+      </c>
+      <c r="F8" s="34">
+        <f>-PL!K13</f>
+        <v/>
+      </c>
+      <c r="G8" s="34">
+        <f>-PL!L13</f>
+        <v/>
+      </c>
+      <c r="H8" s="34">
+        <f>-PL!M13</f>
+        <v/>
+      </c>
+      <c r="I8" s="34">
+        <f>-PL!N13</f>
+        <v/>
+      </c>
+      <c r="J8" s="34">
+        <f>-PL!O13</f>
         <v/>
       </c>
       <c r="L8" s="7" t="inlineStr">
@@ -3519,42 +3579,42 @@
     <row r="9">
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Add: Depreciation &amp; amortisation</t>
+          <t>Less: Capex (PPE + intangibles)</t>
         </is>
       </c>
       <c r="C9" s="34">
-        <f>-PL!H13</f>
+        <f>-('Working Schedules'!H7+'Working Schedules'!H21)</f>
         <v/>
       </c>
       <c r="D9" s="34">
-        <f>-PL!I13</f>
+        <f>-('Working Schedules'!I7+'Working Schedules'!I21)</f>
         <v/>
       </c>
       <c r="E9" s="34">
-        <f>-PL!J13</f>
+        <f>-('Working Schedules'!J7+'Working Schedules'!J21)</f>
         <v/>
       </c>
       <c r="F9" s="34">
-        <f>-PL!K13</f>
+        <f>-('Working Schedules'!K7+'Working Schedules'!K21)</f>
         <v/>
       </c>
       <c r="G9" s="34">
-        <f>-PL!L13</f>
+        <f>-('Working Schedules'!L7+'Working Schedules'!L21)</f>
         <v/>
       </c>
       <c r="H9" s="34">
-        <f>-PL!M13</f>
+        <f>-('Working Schedules'!M7+'Working Schedules'!M21)</f>
         <v/>
       </c>
       <c r="I9" s="34">
-        <f>-PL!N13</f>
+        <f>-('Working Schedules'!N7+'Working Schedules'!N21)</f>
         <v/>
       </c>
       <c r="J9" s="34">
-        <f>-PL!O13</f>
-        <v/>
-      </c>
-      <c r="L9" s="12" t="inlineStr">
+        <f>-('Working Schedules'!O7+'Working Schedules'!O21)</f>
+        <v/>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
         <is>
           <t>WACC</t>
         </is>
@@ -3572,326 +3632,677 @@
     <row r="10">
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Less: Capex (PPE + intangibles)</t>
+          <t>Less: Increase in net working capital</t>
         </is>
       </c>
       <c r="C10" s="34">
-        <f>-('Working Schedules'!H7+'Working Schedules'!H21)</f>
+        <f>-'Working Capital Schedule'!H21</f>
         <v/>
       </c>
       <c r="D10" s="34">
-        <f>-('Working Schedules'!I7+'Working Schedules'!I21)</f>
+        <f>-'Working Capital Schedule'!I21</f>
         <v/>
       </c>
       <c r="E10" s="34">
-        <f>-('Working Schedules'!J7+'Working Schedules'!J21)</f>
+        <f>-'Working Capital Schedule'!J21</f>
         <v/>
       </c>
       <c r="F10" s="34">
-        <f>-('Working Schedules'!K7+'Working Schedules'!K21)</f>
+        <f>-'Working Capital Schedule'!K21</f>
         <v/>
       </c>
       <c r="G10" s="34">
-        <f>-('Working Schedules'!L7+'Working Schedules'!L21)</f>
+        <f>-'Working Capital Schedule'!L21</f>
         <v/>
       </c>
       <c r="H10" s="34">
-        <f>-('Working Schedules'!M7+'Working Schedules'!M21)</f>
+        <f>-'Working Capital Schedule'!M21</f>
         <v/>
       </c>
       <c r="I10" s="34">
-        <f>-('Working Schedules'!N7+'Working Schedules'!N21)</f>
+        <f>-'Working Capital Schedule'!N21</f>
         <v/>
       </c>
       <c r="J10" s="34">
-        <f>-('Working Schedules'!O7+'Working Schedules'!O21)</f>
+        <f>-'Working Capital Schedule'!O21</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Less: Increase in net working capital</t>
-        </is>
-      </c>
-      <c r="C11" s="34">
-        <f>-'Working Capital Schedule'!H21</f>
-        <v/>
-      </c>
-      <c r="D11" s="34">
-        <f>-'Working Capital Schedule'!I21</f>
-        <v/>
-      </c>
-      <c r="E11" s="34">
-        <f>-'Working Capital Schedule'!J21</f>
-        <v/>
-      </c>
-      <c r="F11" s="34">
-        <f>-'Working Capital Schedule'!K21</f>
-        <v/>
-      </c>
-      <c r="G11" s="34">
-        <f>-'Working Capital Schedule'!L21</f>
-        <v/>
-      </c>
-      <c r="H11" s="34">
-        <f>-'Working Capital Schedule'!M21</f>
-        <v/>
-      </c>
-      <c r="I11" s="34">
-        <f>-'Working Capital Schedule'!N21</f>
-        <v/>
-      </c>
-      <c r="J11" s="34">
-        <f>-'Working Capital Schedule'!O21</f>
+      <c r="B11" s="35" t="inlineStr">
+        <is>
+          <t>FCFF</t>
+        </is>
+      </c>
+      <c r="C11" s="36">
+        <f>SUM(C7:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="36">
+        <f>SUM(D7:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="36">
+        <f>SUM(E7:E10)</f>
+        <v/>
+      </c>
+      <c r="F11" s="36">
+        <f>SUM(F7:F10)</f>
+        <v/>
+      </c>
+      <c r="G11" s="36">
+        <f>SUM(G7:G10)</f>
+        <v/>
+      </c>
+      <c r="H11" s="36">
+        <f>SUM(H7:H10)</f>
+        <v/>
+      </c>
+      <c r="I11" s="36">
+        <f>SUM(I7:I10)</f>
+        <v/>
+      </c>
+      <c r="J11" s="36">
+        <f>SUM(J7:J10)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="35" t="inlineStr">
-        <is>
-          <t>Free cash flow to firm (FCFF)</t>
-        </is>
-      </c>
-      <c r="C12" s="36">
-        <f>SUM(C8:C11)</f>
-        <v/>
-      </c>
-      <c r="D12" s="36">
-        <f>SUM(D8:D11)</f>
-        <v/>
-      </c>
-      <c r="E12" s="36">
-        <f>SUM(E8:E11)</f>
-        <v/>
-      </c>
-      <c r="F12" s="36">
-        <f>SUM(F8:F11)</f>
-        <v/>
-      </c>
-      <c r="G12" s="36">
-        <f>SUM(G8:G11)</f>
-        <v/>
-      </c>
-      <c r="H12" s="36">
-        <f>SUM(H8:H11)</f>
-        <v/>
-      </c>
-      <c r="I12" s="36">
-        <f>SUM(I8:I11)</f>
-        <v/>
-      </c>
-      <c r="J12" s="36">
-        <f>SUM(J8:J11)</f>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Discount period</t>
+        </is>
+      </c>
+      <c r="C12" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="47">
+        <f>C12+1</f>
+        <v/>
+      </c>
+      <c r="E12" s="47">
+        <f>D12+1</f>
+        <v/>
+      </c>
+      <c r="F12" s="47">
+        <f>E12+1</f>
+        <v/>
+      </c>
+      <c r="G12" s="47">
+        <f>F12+1</f>
+        <v/>
+      </c>
+      <c r="H12" s="47">
+        <f>G12+1</f>
+        <v/>
+      </c>
+      <c r="I12" s="47">
+        <f>H12+1</f>
+        <v/>
+      </c>
+      <c r="J12" s="47">
+        <f>I12+1</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Discount period</t>
-        </is>
-      </c>
-      <c r="C13" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="47">
-        <f>C13+1</f>
-        <v/>
-      </c>
-      <c r="E13" s="47">
-        <f>D13+1</f>
-        <v/>
-      </c>
-      <c r="F13" s="47">
-        <f>E13+1</f>
-        <v/>
-      </c>
-      <c r="G13" s="47">
-        <f>F13+1</f>
-        <v/>
-      </c>
-      <c r="H13" s="47">
-        <f>G13+1</f>
-        <v/>
-      </c>
-      <c r="I13" s="47">
-        <f>H13+1</f>
-        <v/>
-      </c>
-      <c r="J13" s="47">
-        <f>I13+1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>PV of FCFF</t>
         </is>
       </c>
-      <c r="C14" s="33">
-        <f>C12/(1+$M$9)^C13</f>
-        <v/>
-      </c>
-      <c r="D14" s="33">
-        <f>D12/(1+$M$9)^D13</f>
-        <v/>
-      </c>
-      <c r="E14" s="33">
-        <f>E12/(1+$M$9)^E13</f>
-        <v/>
-      </c>
-      <c r="F14" s="33">
-        <f>F12/(1+$M$9)^F13</f>
-        <v/>
-      </c>
-      <c r="G14" s="33">
-        <f>G12/(1+$M$9)^G13</f>
-        <v/>
-      </c>
-      <c r="H14" s="33">
-        <f>H12/(1+$M$9)^H13</f>
-        <v/>
-      </c>
-      <c r="I14" s="33">
-        <f>I12/(1+$M$9)^I13</f>
-        <v/>
-      </c>
-      <c r="J14" s="33">
-        <f>J12/(1+$M$9)^J13</f>
-        <v/>
-      </c>
+      <c r="C13" s="33">
+        <f>C11/(1+$M$9)^C12</f>
+        <v/>
+      </c>
+      <c r="D13" s="33">
+        <f>D11/(1+$M$9)^D12</f>
+        <v/>
+      </c>
+      <c r="E13" s="33">
+        <f>E11/(1+$M$9)^E12</f>
+        <v/>
+      </c>
+      <c r="F13" s="33">
+        <f>F11/(1+$M$9)^F12</f>
+        <v/>
+      </c>
+      <c r="G13" s="33">
+        <f>G11/(1+$M$9)^G12</f>
+        <v/>
+      </c>
+      <c r="H13" s="33">
+        <f>H11/(1+$M$9)^H12</f>
+        <v/>
+      </c>
+      <c r="I13" s="33">
+        <f>I11/(1+$M$9)^I12</f>
+        <v/>
+      </c>
+      <c r="J13" s="33">
+        <f>J11/(1+$M$9)^J12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>Stage 2 — Fade / convergence (FY2034E–FY2040E): growth &amp; margins converge to steady state</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="n"/>
+      <c r="D15" s="20" t="n"/>
+      <c r="E15" s="20" t="n"/>
+      <c r="F15" s="20" t="n"/>
+      <c r="G15" s="20" t="n"/>
+      <c r="H15" s="20" t="n"/>
+      <c r="I15" s="20" t="n"/>
+      <c r="J15" s="20" t="n"/>
+      <c r="K15" s="20" t="n"/>
+      <c r="L15" s="20" t="n"/>
+      <c r="M15" s="20" t="n"/>
+      <c r="N15" s="20" t="n"/>
+      <c r="O15" s="20" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Valuation summary</t>
-        </is>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>Particulars</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="n">
+        <v>2034</v>
+      </c>
+      <c r="D16" s="23">
+        <f>C16+1</f>
+        <v/>
+      </c>
+      <c r="E16" s="23">
+        <f>D16+1</f>
+        <v/>
+      </c>
+      <c r="F16" s="23">
+        <f>E16+1</f>
+        <v/>
+      </c>
+      <c r="G16" s="23">
+        <f>F16+1</f>
+        <v/>
+      </c>
+      <c r="H16" s="23">
+        <f>G16+1</f>
+        <v/>
+      </c>
+      <c r="I16" s="23">
+        <f>H16+1</f>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Terminal growth rate (g)</t>
-        </is>
-      </c>
-      <c r="C17" s="50" t="n">
-        <v>0.05</v>
+          <t>Revenue growth %</t>
+        </is>
+      </c>
+      <c r="C17" s="25" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="D17" s="25" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E17" s="25" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="F17" s="25" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G17" s="25" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="H17" s="25" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="I17" s="25" t="n">
+        <v>0.055</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Terminal (steady-state) EBIT margin</t>
-        </is>
-      </c>
-      <c r="C18" s="50" t="n">
-        <v>0.1</v>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C18" s="34">
+        <f>PL!O5*(1+C17)</f>
+        <v/>
+      </c>
+      <c r="D18" s="39">
+        <f>C18*(1+D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="39">
+        <f>D18*(1+E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="39">
+        <f>E18*(1+F17)</f>
+        <v/>
+      </c>
+      <c r="G18" s="39">
+        <f>F18*(1+G17)</f>
+        <v/>
+      </c>
+      <c r="H18" s="39">
+        <f>G18*(1+H17)</f>
+        <v/>
+      </c>
+      <c r="I18" s="39">
+        <f>H18*(1+I17)</f>
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Normalised terminal NOPAT</t>
-        </is>
-      </c>
-      <c r="C19" s="39">
-        <f>PL!O5*C18*(1-Assumptions!O47)</f>
-        <v/>
+          <t>EBIT margin %</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G19" s="25" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H19" s="25" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="I19" s="25" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Terminal value (end FY2033)</t>
+          <t>EBIT</t>
         </is>
       </c>
       <c r="C20" s="39">
-        <f>C19*(1+C17)/($M$9-C17)</f>
+        <f>C18*C19</f>
+        <v/>
+      </c>
+      <c r="D20" s="39">
+        <f>D18*D19</f>
+        <v/>
+      </c>
+      <c r="E20" s="39">
+        <f>E18*E19</f>
+        <v/>
+      </c>
+      <c r="F20" s="39">
+        <f>F18*F19</f>
+        <v/>
+      </c>
+      <c r="G20" s="39">
+        <f>G18*G19</f>
+        <v/>
+      </c>
+      <c r="H20" s="39">
+        <f>H18*H19</f>
+        <v/>
+      </c>
+      <c r="I20" s="39">
+        <f>I18*I19</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="7" t="inlineStr">
         <is>
+          <t>Effective tax rate %</t>
+        </is>
+      </c>
+      <c r="C21" s="25" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D21" s="25" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E21" s="25" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F21" s="25" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="G21" s="25" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H21" s="25" t="n">
+        <v>0.2517</v>
+      </c>
+      <c r="I21" s="25" t="n">
+        <v>0.2517</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>NOPAT</t>
+        </is>
+      </c>
+      <c r="C22" s="33">
+        <f>C20*(1-C21)</f>
+        <v/>
+      </c>
+      <c r="D22" s="33">
+        <f>D20*(1-D21)</f>
+        <v/>
+      </c>
+      <c r="E22" s="33">
+        <f>E20*(1-E21)</f>
+        <v/>
+      </c>
+      <c r="F22" s="33">
+        <f>F20*(1-F21)</f>
+        <v/>
+      </c>
+      <c r="G22" s="33">
+        <f>G20*(1-G21)</f>
+        <v/>
+      </c>
+      <c r="H22" s="33">
+        <f>H20*(1-H21)</f>
+        <v/>
+      </c>
+      <c r="I22" s="33">
+        <f>I20*(1-I21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Reinvestment rate % (capex+NWC, net of D&amp;A)</t>
+        </is>
+      </c>
+      <c r="C23" s="25" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="D23" s="25" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E23" s="25" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F23" s="25" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G23" s="25" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="H23" s="25" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="I23" s="25" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="35" t="inlineStr">
+        <is>
+          <t>FCFF</t>
+        </is>
+      </c>
+      <c r="C24" s="36">
+        <f>C22*(1-C23)</f>
+        <v/>
+      </c>
+      <c r="D24" s="36">
+        <f>D22*(1-D23)</f>
+        <v/>
+      </c>
+      <c r="E24" s="36">
+        <f>E22*(1-E23)</f>
+        <v/>
+      </c>
+      <c r="F24" s="36">
+        <f>F22*(1-F23)</f>
+        <v/>
+      </c>
+      <c r="G24" s="36">
+        <f>G22*(1-G23)</f>
+        <v/>
+      </c>
+      <c r="H24" s="36">
+        <f>H22*(1-H23)</f>
+        <v/>
+      </c>
+      <c r="I24" s="36">
+        <f>I22*(1-I23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Discount period</t>
+        </is>
+      </c>
+      <c r="C25" s="47">
+        <f>J12+1</f>
+        <v/>
+      </c>
+      <c r="D25" s="47">
+        <f>C25+1</f>
+        <v/>
+      </c>
+      <c r="E25" s="47">
+        <f>D25+1</f>
+        <v/>
+      </c>
+      <c r="F25" s="47">
+        <f>E25+1</f>
+        <v/>
+      </c>
+      <c r="G25" s="47">
+        <f>F25+1</f>
+        <v/>
+      </c>
+      <c r="H25" s="47">
+        <f>G25+1</f>
+        <v/>
+      </c>
+      <c r="I25" s="47">
+        <f>H25+1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>PV of FCFF</t>
+        </is>
+      </c>
+      <c r="C26" s="33">
+        <f>C24/(1+$M$9)^C25</f>
+        <v/>
+      </c>
+      <c r="D26" s="33">
+        <f>D24/(1+$M$9)^D25</f>
+        <v/>
+      </c>
+      <c r="E26" s="33">
+        <f>E24/(1+$M$9)^E25</f>
+        <v/>
+      </c>
+      <c r="F26" s="33">
+        <f>F24/(1+$M$9)^F25</f>
+        <v/>
+      </c>
+      <c r="G26" s="33">
+        <f>G24/(1+$M$9)^G25</f>
+        <v/>
+      </c>
+      <c r="H26" s="33">
+        <f>H24/(1+$M$9)^H25</f>
+        <v/>
+      </c>
+      <c r="I26" s="33">
+        <f>I24/(1+$M$9)^I25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="19" t="inlineStr">
+        <is>
+          <t>Valuation summary</t>
+        </is>
+      </c>
+      <c r="C28" s="20" t="n"/>
+      <c r="D28" s="20" t="n"/>
+      <c r="E28" s="20" t="n"/>
+      <c r="F28" s="20" t="n"/>
+      <c r="G28" s="20" t="n"/>
+      <c r="H28" s="20" t="n"/>
+      <c r="I28" s="20" t="n"/>
+      <c r="J28" s="20" t="n"/>
+      <c r="K28" s="20" t="n"/>
+      <c r="L28" s="20" t="n"/>
+      <c r="M28" s="20" t="n"/>
+      <c r="N28" s="20" t="n"/>
+      <c r="O28" s="20" t="n"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Terminal growth rate (g)</t>
+        </is>
+      </c>
+      <c r="C29" s="50" t="n">
+        <v>0.055</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Sum of PV — Stage 1 (FY26-33)</t>
+        </is>
+      </c>
+      <c r="C30" s="39">
+        <f>SUM(C13:J13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Sum of PV — Stage 2 (FY34-40)</t>
+        </is>
+      </c>
+      <c r="C31" s="39">
+        <f>SUM(C26:I26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Terminal value (end FY2040)</t>
+        </is>
+      </c>
+      <c r="C32" s="39">
+        <f>I24*(1+C29)/($M$9-C29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="7" t="inlineStr">
+        <is>
           <t>PV of terminal value</t>
         </is>
       </c>
-      <c r="C21" s="39">
-        <f>C20/(1+$M$9)^J13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>Sum of PV of explicit FCFF</t>
-        </is>
-      </c>
-      <c r="C22" s="39">
-        <f>SUM(C14:J14)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="12" t="inlineStr">
+      <c r="C33" s="39">
+        <f>C32/(1+$M$9)^I25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>Enterprise value (EV)</t>
         </is>
       </c>
-      <c r="C23" s="33">
-        <f>C21+C22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="7" t="inlineStr">
+      <c r="C34" s="33">
+        <f>C30+C31+C33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>Less: net debt (FY2025)</t>
         </is>
       </c>
-      <c r="C24" s="34">
+      <c r="C35" s="34">
         <f>-(BS!G13+BS!G21+BS!G14+BS!G22-BS!G43)</f>
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="12" t="inlineStr">
+    <row r="36">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>Equity value</t>
         </is>
       </c>
-      <c r="C25" s="33">
-        <f>C23+C24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="7" t="inlineStr">
+      <c r="C36" s="33">
+        <f>C34+C35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>Shares outstanding (m)</t>
         </is>
       </c>
-      <c r="C26" s="27" t="n">
+      <c r="C37" s="27" t="n">
         <v>372</v>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="35" t="inlineStr">
+    <row r="38">
+      <c r="B38" s="35" t="inlineStr">
         <is>
           <t>Value per share (INR)</t>
         </is>
       </c>
-      <c r="C27" s="53">
-        <f>C25/C26</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>Note: Ather is in an investment / pre-profit phase, so explicit-period FCFF is negative and value is dominated by the terminal value, which is built on a normalised steady-state EBIT margin (input) rather than the still-maturing FY2033 margin. The DCF is highly sensitive to WACC, terminal growth and terminal margin and should be read alongside relative valuation (EV/Sales) and the Base/Bull/Bear scenarios.</t>
+      <c r="C38" s="53">
+        <f>C36/C37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>% of value in terminal value</t>
+        </is>
+      </c>
+      <c r="C40" s="54">
+        <f>C33/C34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" ht="58" customHeight="1">
+      <c r="B42" s="55" t="inlineStr">
+        <is>
+          <t>Note: 3-stage FCFF. Stage 1 is the detailed model. Stage 2 lets growth fade and EBIT margin ramp to a mature ~15% before the terminal value is struck on a steady-state business (taxed NOPAT, reinvestment for growth). This is more rigorous than a single-period terminal off the still-maturing FY2033 — note the terminal value now correctly reflects tax and reinvestment. Highly sensitive to WACC, g, terminal margin and the fade path; read with the Relative Valuation and the Scenarios switch.</t>
         </is>
       </c>
     </row>
@@ -3932,64 +4343,64 @@
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
-      <c r="B3" s="54" t="inlineStr">
+      <c r="B3" s="55" t="inlineStr">
         <is>
           <t>Peer market data indicative, as of ~Jun-2026 (public sources: NSE/BSE, stockanalysis, dhan, companies-marketcap). Figures in INR crore unless stated. 1 cr = 10 INR m.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="B5" s="55" t="inlineStr">
+      <c r="B5" s="56" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="C5" s="55" t="inlineStr">
+      <c r="C5" s="56" t="inlineStr">
         <is>
           <t>Mkt cap (cr)</t>
         </is>
       </c>
-      <c r="D5" s="55" t="inlineStr">
+      <c r="D5" s="56" t="inlineStr">
         <is>
           <t>Net debt (cr)</t>
         </is>
       </c>
-      <c r="E5" s="55" t="inlineStr">
+      <c r="E5" s="56" t="inlineStr">
         <is>
           <t>EV (cr)</t>
         </is>
       </c>
-      <c r="F5" s="55" t="inlineStr">
+      <c r="F5" s="56" t="inlineStr">
         <is>
           <t>Revenue (cr)</t>
         </is>
       </c>
-      <c r="G5" s="55" t="inlineStr">
+      <c r="G5" s="56" t="inlineStr">
         <is>
           <t>EBITDA (cr)</t>
         </is>
       </c>
-      <c r="H5" s="55" t="inlineStr">
+      <c r="H5" s="56" t="inlineStr">
         <is>
           <t>PAT (cr)</t>
         </is>
       </c>
-      <c r="I5" s="55" t="inlineStr">
+      <c r="I5" s="56" t="inlineStr">
         <is>
           <t>EV/Sales</t>
         </is>
       </c>
-      <c r="J5" s="55" t="inlineStr">
+      <c r="J5" s="56" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="K5" s="55" t="inlineStr">
+      <c r="K5" s="56" t="inlineStr">
         <is>
           <t>P/E</t>
         </is>
       </c>
-      <c r="L5" s="55" t="inlineStr">
+      <c r="L5" s="56" t="inlineStr">
         <is>
           <t>EBITDA %</t>
         </is>
@@ -4007,7 +4418,7 @@
       <c r="D6" s="28" t="n">
         <v>2000</v>
       </c>
-      <c r="E6" s="56">
+      <c r="E6" s="57">
         <f>C6+D6</f>
         <v/>
       </c>
@@ -4049,7 +4460,7 @@
       <c r="D7" s="28" t="n">
         <v>-15000</v>
       </c>
-      <c r="E7" s="56">
+      <c r="E7" s="57">
         <f>C7+D7</f>
         <v/>
       </c>
@@ -4091,7 +4502,7 @@
       <c r="D8" s="28" t="n">
         <v>-8000</v>
       </c>
-      <c r="E8" s="56">
+      <c r="E8" s="57">
         <f>C8+D8</f>
         <v/>
       </c>
@@ -4133,7 +4544,7 @@
       <c r="D9" s="28" t="n">
         <v>-16000</v>
       </c>
-      <c r="E9" s="56">
+      <c r="E9" s="57">
         <f>C9+D9</f>
         <v/>
       </c>
@@ -4175,7 +4586,7 @@
       <c r="D10" s="28" t="n">
         <v>-2000</v>
       </c>
-      <c r="E10" s="56">
+      <c r="E10" s="57">
         <f>C10+D10</f>
         <v/>
       </c>
@@ -4217,7 +4628,7 @@
       <c r="D11" s="28" t="n">
         <v>150</v>
       </c>
-      <c r="E11" s="56">
+      <c r="E11" s="57">
         <f>C11+D11</f>
         <v/>
       </c>
@@ -4253,15 +4664,15 @@
           <t>Legacy 2W OEM median (TVS/Bajaj/Hero/Eicher)</t>
         </is>
       </c>
-      <c r="I13" s="57">
+      <c r="I13" s="58">
         <f>MEDIAN(I6:I9)</f>
         <v/>
       </c>
-      <c r="J13" s="57">
+      <c r="J13" s="58">
         <f>MEDIAN(J6:J9)</f>
         <v/>
       </c>
-      <c r="K13" s="57">
+      <c r="K13" s="58">
         <f>MEDIAN(K6:K9)</f>
         <v/>
       </c>
@@ -4272,7 +4683,7 @@
           <t>EV pure-play reference (Ola Electric)</t>
         </is>
       </c>
-      <c r="I14" s="57">
+      <c r="I14" s="58">
         <f>I10</f>
         <v/>
       </c>
@@ -4335,22 +4746,22 @@
           <t>Scenario</t>
         </is>
       </c>
-      <c r="C21" s="58" t="inlineStr">
+      <c r="C21" s="59" t="inlineStr">
         <is>
           <t>EV/Sales (x)</t>
         </is>
       </c>
-      <c r="D21" s="58" t="inlineStr">
+      <c r="D21" s="59" t="inlineStr">
         <is>
           <t>Implied EV (cr)</t>
         </is>
       </c>
-      <c r="E21" s="58" t="inlineStr">
+      <c r="E21" s="59" t="inlineStr">
         <is>
           <t>Implied equity (cr)</t>
         </is>
       </c>
-      <c r="F21" s="58" t="inlineStr">
+      <c r="F21" s="59" t="inlineStr">
         <is>
           <t>Implied price (INR)</t>
         </is>
@@ -4362,18 +4773,18 @@
           <t>Conservative (3.0x)</t>
         </is>
       </c>
-      <c r="C22" s="59" t="n">
+      <c r="C22" s="60" t="n">
         <v>3</v>
       </c>
-      <c r="D22" s="56">
+      <c r="D22" s="57">
         <f>C22*$C$17</f>
         <v/>
       </c>
-      <c r="E22" s="56">
+      <c r="E22" s="57">
         <f>D22-$C$18</f>
         <v/>
       </c>
-      <c r="F22" s="60">
+      <c r="F22" s="61">
         <f>E22*10/$C$19</f>
         <v/>
       </c>
@@ -4384,18 +4795,18 @@
           <t>Base (4.5x)</t>
         </is>
       </c>
-      <c r="C23" s="59" t="n">
+      <c r="C23" s="60" t="n">
         <v>4.5</v>
       </c>
-      <c r="D23" s="56">
+      <c r="D23" s="57">
         <f>C23*$C$17</f>
         <v/>
       </c>
-      <c r="E23" s="56">
+      <c r="E23" s="57">
         <f>D23-$C$18</f>
         <v/>
       </c>
-      <c r="F23" s="60">
+      <c r="F23" s="61">
         <f>E23*10/$C$19</f>
         <v/>
       </c>
@@ -4406,18 +4817,18 @@
           <t>Bull (6.0x)</t>
         </is>
       </c>
-      <c r="C24" s="59" t="n">
+      <c r="C24" s="60" t="n">
         <v>6</v>
       </c>
-      <c r="D24" s="56">
+      <c r="D24" s="57">
         <f>C24*$C$17</f>
         <v/>
       </c>
-      <c r="E24" s="56">
+      <c r="E24" s="57">
         <f>D24-$C$18</f>
         <v/>
       </c>
-      <c r="F24" s="60">
+      <c r="F24" s="61">
         <f>E24*10/$C$19</f>
         <v/>
       </c>
@@ -4448,8 +4859,8 @@
           <t>DCF — Base case (INR/share)</t>
         </is>
       </c>
-      <c r="C28" s="61">
-        <f>DCF!C27</f>
+      <c r="C28" s="62">
+        <f>DCF!C38</f>
         <v/>
       </c>
     </row>
@@ -4459,7 +4870,7 @@
           <t>Relative — conservative to bull (INR/share)</t>
         </is>
       </c>
-      <c r="C29" s="60">
+      <c r="C29" s="61">
         <f>F22</f>
         <v/>
       </c>
@@ -4474,7 +4885,7 @@
           <t>Current market price (INR/share)</t>
         </is>
       </c>
-      <c r="C30" s="62" t="n">
+      <c r="C30" s="63" t="n">
         <v>990</v>
       </c>
     </row>
@@ -4484,13 +4895,13 @@
           <t>Implied market EV/Sales on FY25 revenue (x)</t>
         </is>
       </c>
-      <c r="C31" s="63">
+      <c r="C31" s="64">
         <f>I11</f>
         <v/>
       </c>
     </row>
     <row r="33" ht="58" customHeight="1">
-      <c r="B33" s="54" t="inlineStr">
+      <c r="B33" s="55" t="inlineStr">
         <is>
           <t>Read-through: Ather trades at a steep premium to legacy 2W OEMs and to Ola Electric on EV/Sales, so the market is already pricing in strong volume growth and a sharp margin ramp. On a conservative DCF and on peer-based EV/Sales, the stock screens expensive unless one underwrites the bull-case volumes and terminal margins. Use this alongside the DCF and the Scenarios switch. Indicative, not investment advice.</t>
         </is>
@@ -4523,112 +4934,112 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="B4" s="64" t="inlineStr">
+      <c r="B4" s="65" t="inlineStr">
         <is>
           <t>Company snapshot</t>
         </is>
       </c>
     </row>
     <row r="5" ht="60" customHeight="1">
-      <c r="B5" s="65" t="inlineStr">
+      <c r="B5" s="66" t="inlineStr">
         <is>
           <t>Ather Energy Ltd (Bengaluru; incorporated 2013) designs and manufactures premium smart electric scooters (450 series, Rizta) and runs the AtherStack software and Ather Grid charging ecosystem. It listed on NSE/BSE in May 2025. Ather prepares STANDALONE financial statements only — it has no subsidiaries, so no consolidated statements exist; standalone is therefore the consolidated-equivalent used here.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="B6" s="64" t="inlineStr">
+      <c r="B6" s="65" t="inlineStr">
         <is>
           <t>Operating performance</t>
         </is>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1">
-      <c r="B7" s="65" t="inlineStr">
+      <c r="B7" s="66" t="inlineStr">
         <is>
           <t>Revenue grew from INR 798m (FY21) to INR 22,550m (FY25); FY25 revenue +29% YoY. The company remains loss-making (FY25 PAT INR -8,123m) but gross margin inflected sharply to ~16.8% in FY25 (from ~7% FY24) on scale, the Rizta launch and falling battery costs. Vehicle sales are ~88% of revenue; software, accessories, charging and service make up the balance and are higher-margin, recurring streams.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="B8" s="64" t="inlineStr">
+      <c r="B8" s="65" t="inlineStr">
         <is>
           <t>Volumes, ASP &amp; market share</t>
         </is>
       </c>
     </row>
     <row r="9" ht="60" customHeight="1">
-      <c r="B9" s="65" t="inlineStr">
+      <c r="B9" s="66" t="inlineStr">
         <is>
           <t>FY25 deliveries ~1.65 lakh units; revenue per vehicle ~INR 1.28 lakh (down from ~1.43 lakh FY24 and ~1.56 lakh FY23 as the cheaper Rizta lifted mix). Ather's E2W market share rose from ~13-14% (FY25) to ~18.7% by Mar-2026; retail network expanded from 351 outlets (Mar-25) toward ~700 (FY26). Source: Vahan / ETAuto / Autocar India / Storyboard18.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="B10" s="64" t="inlineStr">
+      <c r="B10" s="65" t="inlineStr">
         <is>
           <t>Industry &amp; demand drivers</t>
         </is>
       </c>
     </row>
     <row r="11" ht="60" customHeight="1">
-      <c r="B11" s="65" t="inlineStr">
+      <c r="B11" s="66" t="inlineStr">
         <is>
           <t>India electric two-wheeler volumes (~1.1-1.2m in FY25) are forecast to grow ~26-28% CAGR to 2034 (IMARC/Renub/TechSci). E2W penetration of the ~19m-unit 2W market is ~6-7% today and is projected at ~30% by 2030 (Kearney) and up to ~40% by FY31 in Ather's optimistic case. PM E-DRIVE (successor to FAME-II), 5% GST on EVs, state EV policies and PLI for cell manufacturing support demand and localisation.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="B12" s="64" t="inlineStr">
+      <c r="B12" s="65" t="inlineStr">
         <is>
           <t>Battery cost trend (key margin lever)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="45" customHeight="1">
-      <c r="B13" s="65" t="inlineStr">
+      <c r="B13" s="66" t="inlineStr">
         <is>
           <t>Lithium-ion pack prices fell ~8% to ~USD 108/kWh in 2025 and are forecast at ~USD 105/kWh in 2026, declining toward ~USD 80-90/kWh by 2030 (BloombergNEF, Dec-2025), aided by cell overcapacity and an ~84% lithium price correction. Batteries are Ather's largest input cost, so this is a structural gross-margin tailwind.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
-      <c r="B14" s="64" t="inlineStr">
+      <c r="B14" s="65" t="inlineStr">
         <is>
           <t>Competition</t>
         </is>
       </c>
     </row>
     <row r="15" ht="60" customHeight="1">
-      <c r="B15" s="65" t="inlineStr">
+      <c r="B15" s="66" t="inlineStr">
         <is>
           <t>Top E2W OEMs (CY2025 / early-2026 Vahan): TVS Motor ~24%, Bajaj Auto ~22%, Ather ~13-18%, with Ola Electric's share collapsing (24.8% Jan-25 to &lt;6% Jan-26), plus Hero/Greaves. TVS and Bajaj are profitable legacy OEMs with large ICE dealer networks; Ola and Ather are pure-play EV challengers still investing for scale. Ather differentiates on software, design and a premium brand.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="B16" s="64" t="inlineStr">
+      <c r="B16" s="65" t="inlineStr">
         <is>
           <t>Capital &amp; capacity</t>
         </is>
       </c>
     </row>
     <row r="17" ht="45" customHeight="1">
-      <c r="B17" s="65" t="inlineStr">
+      <c r="B17" s="66" t="inlineStr">
         <is>
           <t>The IPO raised a fresh issue of ~INR 2,626 cr (~26,260m), used for the new Maharashtra plant (Factory-3, tripling capacity), R&amp;D, debt repayment and marketing. Post-IPO shares outstanding ~372m. Large accumulated tax losses (&gt;INR 40,000m) shield taxable income across the forecast horizon (statutory rate 25.17%).</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="B18" s="64" t="inlineStr">
+      <c r="B18" s="65" t="inlineStr">
         <is>
           <t>Sources</t>
         </is>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
-      <c r="B19" s="66" t="inlineStr">
+      <c r="B19" s="67" t="inlineStr">
         <is>
           <t>BloombergNEF battery price survey (Dec-2025); SIAM / Vahan registration data; ETAuto, Economic Times, Moneycontrol, Autocar India, Storyboard18, Angel One, Financial Express; IMARC / Renub / TechSci / Kearney industry reports; Ather Energy Annual Reports FY2021-FY2025 (standalone financial statements). Content paraphrased / summarised for licensing compliance.</t>
         </is>
@@ -4661,140 +5072,140 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="B4" s="67" t="inlineStr">
+      <c r="B4" s="68" t="inlineStr">
         <is>
           <t>1. Purpose &amp; scope</t>
         </is>
       </c>
     </row>
     <row r="5" ht="60" customHeight="1">
-      <c r="B5" s="65" t="inlineStr">
+      <c r="B5" s="66" t="inlineStr">
         <is>
           <t>Fully-linked, driver-based operating model and DCF for Ather Energy Ltd. History FY2021-FY2025; forecast FY2026E-FY2033E (8 years). All figures INR millions unless stated. Built to mirror the supplied United Spirits template's structure, colour coding and philosophy. Colour key: BLUE = hardcoded input, GREEN = link/reference to another sheet, BLACK = in-sheet calculation.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="B6" s="67" t="inlineStr">
+      <c r="B6" s="68" t="inlineStr">
         <is>
           <t>2. Data basis (consolidated vs standalone)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="105" customHeight="1">
-      <c r="B7" s="65" t="inlineStr">
+      <c r="B7" s="66" t="inlineStr">
         <is>
           <t>Ather has no subsidiaries and files only STANDALONE Ind AS financial statements; no consolidated statements exist, so standalone is used as the consolidated-equivalent. FY2021/22/24/25 are taken directly from the annual reports in the repository. FY2023's annual reports in the repo are image-only (no text layer); FY2023 was therefore reconstructed from reliable public sources (Economic Times/Moneycontrol: revenue INR 17,836m, total expenses INR 26,706m, net loss INR 8,645m, D&amp;A INR 1,128m) and from anchors verified in the FY2025 report (1-Apr-2023 reserves INR 6,131m; opening borrowings/lease; opening cash INR 826m; FY23 inventory INR 2,574m). FY2023 sub-line splits are estimates that reconcile exactly to the verified totals.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="B8" s="67" t="inlineStr">
+      <c r="B8" s="68" t="inlineStr">
         <is>
           <t>3. Revenue methodology</t>
         </is>
       </c>
     </row>
     <row r="9" ht="90" customHeight="1">
-      <c r="B9" s="65" t="inlineStr">
+      <c r="B9" s="66" t="inlineStr">
         <is>
           <t>Driver-based: vehicle revenue = unit volumes x ASP. Volume growth is set on the Scenarios sheet (Base/Bull/Bear) reflecting E2W market growth plus Ather share gains, tapering over time. ASP reflects the recent Rizta-led mix dip then modest premiumisation. Accessories, software/connectivity and charging are forecast as a % of vehicle revenue (higher-margin recurring streams broken out prospectively); service grows with the installed fleet. Historically these streams were bundled into product/service revenue per Note 20, so a small step-up appears in FY2026.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="B10" s="67" t="inlineStr">
+      <c r="B10" s="68" t="inlineStr">
         <is>
           <t>4. Cost, margin &amp; operating leverage</t>
         </is>
       </c>
     </row>
     <row r="11" ht="75" customHeight="1">
-      <c r="B11" s="65" t="inlineStr">
+      <c r="B11" s="66" t="inlineStr">
         <is>
           <t>Gross margin (Scenarios) expands from ~18% (FY26) to ~28% (FY33) on falling battery costs, scale, localisation/PLI and mix. Employee and other operating expenses are forecast as a declining % of sales, capturing operating leverage as a largely fixed cost base is spread over a fast-growing top line. The model reaches EBITDA breakeven around FY2030 and approaches PAT breakeven by FY2032-FY2033 — a realistic path, neither over-optimistic nor over-pessimistic.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="B12" s="67" t="inlineStr">
+      <c r="B12" s="68" t="inlineStr">
         <is>
           <t>5. Schedules</t>
         </is>
       </c>
     </row>
     <row r="13" ht="75" customHeight="1">
-      <c r="B13" s="65" t="inlineStr">
+      <c r="B13" s="66" t="inlineStr">
         <is>
           <t>PPE, ROU (leases) and intangibles use opening + additions - depreciation/amortisation roll-forwards (capex and additions driven off revenue). Depreciation uses a straight-line life with a half-year convention on additions. Borrowings and leases use opening + net movement roll-forwards with interest on opening balances feeding the finance-cost schedule. A tax schedule tracks carry-forward losses (&gt;INR 40,000m) which keep cash tax at nil across the forecast.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
-      <c r="B14" s="67" t="inlineStr">
+      <c r="B14" s="68" t="inlineStr">
         <is>
           <t>6. Integration &amp; balancing</t>
         </is>
       </c>
     </row>
     <row r="15" ht="75" customHeight="1">
-      <c r="B15" s="65" t="inlineStr">
+      <c r="B15" s="66" t="inlineStr">
         <is>
           <t>The three statements are fully linked with no circular references (interest income/expense use opening balances). The model is FULLY ARTICULATED: every balance-sheet line is forecast from a driver and cash is the genuine output of the cash-flow statement, so the balance sheet balances by accounting identity (no balancing plug). The Error Checks sheet confirms balance-sheet balancing, cash-flow reconciliation, beginning/ending balances and all roll-forwards return PASS for every year.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="B16" s="67" t="inlineStr">
+      <c r="B16" s="68" t="inlineStr">
         <is>
           <t>7. Valuation</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1">
-      <c r="B17" s="65" t="inlineStr">
-        <is>
-          <t>An FCFF DCF discounts unlevered free cash flow at a CAPM-based WACC (Rf 6.8%, ERP 5.2%, beta 1.15 -&gt; ~12.8%), with a 5% terminal growth rate. Because Ather is pre-profit, early FCFF is negative and most value sits in the terminal year; the DCF should be read alongside relative valuation (EV/Sales) and the Base/Bull/Bear scenarios.</t>
+    <row r="17" ht="105" customHeight="1">
+      <c r="B17" s="66" t="inlineStr">
+        <is>
+          <t>A 3-stage FCFF DCF: Stage 1 is the explicit detailed model (FY2026-FY2033); Stage 2 (FY2034-FY2040) lets revenue growth fade and the EBIT margin ramp to a mature ~15% with taxed NOPAT and reinvestment for growth; the terminal value is then struck on a genuine steady state. Discounted at a CAPM-based WACC (Rf 6.8%, ERP 5.2%, beta 1.15 -&gt; ~12.8%) with ~5.5% terminal growth. This horizon (to FY2040) is appropriate because Ather only reaches EBITDA breakeven around FY2030 and PAT breakeven around FY2032-FY2033 — an 8-year cut-off would strike the terminal value on a still-immature, near-breakeven business. The DCF remains conservative versus the market price; read it alongside the Relative Valuation (EV/Sales) and the Base/Bull/Bear scenarios.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="B18" s="67" t="inlineStr">
+      <c r="B18" s="68" t="inlineStr">
         <is>
           <t>8. Key risks</t>
         </is>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
-      <c r="B19" s="65" t="inlineStr">
+      <c r="B19" s="66" t="inlineStr">
         <is>
           <t>Demand/competition: aggressive pricing by Ola, TVS, Bajaj could cap volumes/ASP and margins. Margin: slower battery-cost decline or input inflation. Execution: Factory-3 ramp and capex discipline. Funding: the model shows cash thinning by FY2033 — a further capital raise or faster profitability may be required. Policy: changes to PM E-DRIVE/GST incentives. Technology: rare-earth magnet supply and battery-chemistry shifts.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
-      <c r="B20" s="67" t="inlineStr">
+      <c r="B20" s="68" t="inlineStr">
         <is>
           <t>9. Limitations</t>
         </is>
       </c>
     </row>
     <row r="21" ht="60" customHeight="1">
-      <c r="B21" s="65" t="inlineStr">
+      <c r="B21" s="66" t="inlineStr">
         <is>
           <t>FY2023 sub-line items are reconstructed (totals verified). Forecasts are scenario-based judgements, not guidance. Other non-current/other current items are modelled as ratios of sales. The DCF is sensitive to WACC and terminal growth (a sensitivity grid can be layered on). This model is for analytical/educational purposes and is not investment advice.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
-      <c r="B22" s="67" t="inlineStr">
+      <c r="B22" s="68" t="inlineStr">
         <is>
           <t>10. How to use</t>
         </is>
       </c>
     </row>
     <row r="23" ht="45" customHeight="1">
-      <c r="B23" s="65" t="inlineStr">
+      <c r="B23" s="66" t="inlineStr">
         <is>
           <t>Change the single Scenarios!F4 switch (1=Base, 2=Bull, 3=Bear) to flex volume growth and gross margin across the whole model. All other assumptions live on the Assumptions sheet (each with a Source and a plain-language Reason). Inputs are blue; do not type over green links or black formulas.</t>
         </is>

</xml_diff>